<commit_message>
auto: 更新 Swing Pattern (US) 2026-08-31
</commit_message>
<xml_diff>
--- a/US_Swing_Pattern.xlsx
+++ b/US_Swing_Pattern.xlsx
@@ -8983,7 +8983,7 @@
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>136.98</v>
+        <v>136.38</v>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
@@ -8994,7 +8994,7 @@
         <v>1.4</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>-2.5</v>
+        <v>-2.9</v>
       </c>
       <c r="G124" s="2" t="n">
         <v>81.39</v>
@@ -9014,26 +9014,28 @@
       <c r="R124" s="2" t="inlineStr"/>
       <c r="S124" s="2" t="inlineStr"/>
       <c r="T124" s="2" t="inlineStr"/>
-      <c r="U124" s="2" t="n">
-        <v>1</v>
+      <c r="U124" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="V124" s="2" t="inlineStr"/>
       <c r="W124" s="2" t="inlineStr"/>
       <c r="X124" s="2" t="inlineStr"/>
       <c r="Y124" s="2" t="n">
-        <v>20.06</v>
+        <v>19.95</v>
       </c>
       <c r="Z124" s="2" t="n">
-        <v>-2.47</v>
+        <v>-2.89</v>
       </c>
       <c r="AA124" s="2" t="n">
-        <v>-2.38</v>
+        <v>-2.81</v>
       </c>
       <c r="AB124" s="2" t="n">
-        <v>-1.78</v>
+        <v>-2.21</v>
       </c>
       <c r="AC124" s="2" t="n">
-        <v>-4.78</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="125">
@@ -11954,7 +11956,7 @@
         </is>
       </c>
       <c r="C167" s="2" t="n">
-        <v>308.98</v>
+        <v>307.82</v>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
@@ -11965,10 +11967,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="F167" s="2" t="n">
-        <v>30.9</v>
+        <v>30.4</v>
       </c>
       <c r="G167" s="2" t="n">
-        <v>106.81</v>
+        <v>105.79</v>
       </c>
       <c r="H167" s="2" t="inlineStr"/>
       <c r="I167" s="2" t="inlineStr"/>
@@ -11986,7 +11988,7 @@
       <c r="O167" s="2" t="inlineStr"/>
       <c r="P167" s="2" t="inlineStr"/>
       <c r="Q167" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R167" s="2" t="inlineStr"/>
       <c r="S167" s="2" t="inlineStr"/>
@@ -11998,19 +12000,19 @@
       <c r="W167" s="2" t="inlineStr"/>
       <c r="X167" s="2" t="inlineStr"/>
       <c r="Y167" s="2" t="n">
-        <v>23.36</v>
+        <v>23.24</v>
       </c>
       <c r="Z167" s="2" t="n">
-        <v>8.58</v>
+        <v>8.17</v>
       </c>
       <c r="AA167" s="2" t="n">
-        <v>9.24</v>
+        <v>8.83</v>
       </c>
       <c r="AB167" s="2" t="n">
-        <v>3.73</v>
+        <v>3.32</v>
       </c>
       <c r="AC167" s="2" t="n">
-        <v>17.52</v>
+        <v>17.12</v>
       </c>
     </row>
     <row r="168">
@@ -19642,30 +19644,24 @@
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="E279" s="2" t="n">
-        <v>-3.16</v>
+        <v>2.53</v>
       </c>
       <c r="F279" s="2" t="n">
-        <v>-41.2</v>
+        <v>9.4</v>
       </c>
       <c r="G279" s="2" t="n">
-        <v>-19.42</v>
-      </c>
-      <c r="H279" s="2" t="inlineStr">
-        <is>
-          <t>底背离</t>
-        </is>
-      </c>
+        <v>34.95</v>
+      </c>
+      <c r="H279" s="2" t="inlineStr"/>
       <c r="I279" s="2" t="inlineStr"/>
       <c r="J279" s="2" t="inlineStr"/>
       <c r="K279" s="2" t="inlineStr"/>
       <c r="L279" s="2" t="inlineStr"/>
-      <c r="M279" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M279" s="2" t="inlineStr"/>
       <c r="N279" s="2" t="inlineStr"/>
       <c r="O279" s="2" t="inlineStr"/>
       <c r="P279" s="2" t="inlineStr"/>
@@ -19680,25 +19676,23 @@
       <c r="U279" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="V279" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="V279" s="2" t="inlineStr"/>
       <c r="W279" s="2" t="inlineStr"/>
       <c r="X279" s="2" t="inlineStr"/>
       <c r="Y279" s="2" t="n">
-        <v>-33.44</v>
+        <v>43.28</v>
       </c>
       <c r="Z279" s="2" t="n">
-        <v>-43.96</v>
+        <v>7.47</v>
       </c>
       <c r="AA279" s="2" t="n">
-        <v>-41.45</v>
+        <v>12.1</v>
       </c>
       <c r="AB279" s="2" t="n">
-        <v>-1.02</v>
+        <v>-3.19</v>
       </c>
       <c r="AC279" s="2" t="n">
-        <v>-2.37</v>
+        <v>-8.289999999999999</v>
       </c>
     </row>
     <row r="280">

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (US) 2026-09-01
</commit_message>
<xml_diff>
--- a/US_Swing_Pattern.xlsx
+++ b/US_Swing_Pattern.xlsx
@@ -8574,7 +8574,7 @@
         <v>4.62</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="G118" s="2" t="n">
         <v>62.56</v>
@@ -8605,19 +8605,19 @@
       <c r="W118" s="2" t="inlineStr"/>
       <c r="X118" s="2" t="inlineStr"/>
       <c r="Y118" s="2" t="n">
-        <v>50.72</v>
+        <v>50.94</v>
       </c>
       <c r="Z118" s="2" t="n">
-        <v>13.46</v>
+        <v>13.23</v>
       </c>
       <c r="AA118" s="2" t="n">
-        <v>17.62</v>
+        <v>17.39</v>
       </c>
       <c r="AB118" s="2" t="n">
-        <v>-2.93</v>
+        <v>-3.24</v>
       </c>
       <c r="AC118" s="2" t="n">
-        <v>-1.27</v>
+        <v>-1.61</v>
       </c>
     </row>
     <row r="119">
@@ -10154,10 +10154,10 @@
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>-9.199999999999999</v>
+        <v>-9.4</v>
       </c>
       <c r="G141" s="2" t="n">
         <v>12.41</v>
@@ -10188,19 +10188,19 @@
       <c r="W141" s="2" t="inlineStr"/>
       <c r="X141" s="2" t="inlineStr"/>
       <c r="Y141" s="2" t="n">
-        <v>12.97</v>
+        <v>12.91</v>
       </c>
       <c r="Z141" s="2" t="n">
-        <v>-11.57</v>
+        <v>-11.81</v>
       </c>
       <c r="AA141" s="2" t="n">
-        <v>-8.32</v>
+        <v>-8.56</v>
       </c>
       <c r="AB141" s="2" t="n">
-        <v>-4.32</v>
+        <v>-4.55</v>
       </c>
       <c r="AC141" s="2" t="n">
-        <v>-5.79</v>
+        <v>-6.02</v>
       </c>
     </row>
     <row r="142">
@@ -35455,7 +35455,7 @@
         <v>1.15</v>
       </c>
       <c r="F511" s="2" t="n">
-        <v>-1.1</v>
+        <v>-1.6</v>
       </c>
       <c r="G511" s="2" t="n">
         <v>10.19</v>
@@ -35480,19 +35480,19 @@
       <c r="W511" s="2" t="inlineStr"/>
       <c r="X511" s="2" t="inlineStr"/>
       <c r="Y511" s="2" t="n">
-        <v>16.58</v>
+        <v>16.98</v>
       </c>
       <c r="Z511" s="2" t="n">
-        <v>-5.96</v>
+        <v>-6.25</v>
       </c>
       <c r="AA511" s="2" t="n">
-        <v>-1.67</v>
+        <v>-1.97</v>
       </c>
       <c r="AB511" s="2" t="n">
-        <v>-2.79</v>
+        <v>-3.21</v>
       </c>
       <c r="AC511" s="2" t="n">
-        <v>-3.6</v>
+        <v>-4.05</v>
       </c>
     </row>
     <row r="512">

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (US) 2026-09-07
</commit_message>
<xml_diff>
--- a/US_Swing_Pattern.xlsx
+++ b/US_Swing_Pattern.xlsx
@@ -1774,9 +1774,7 @@
         <v>1</v>
       </c>
       <c r="R18" s="2" t="inlineStr"/>
-      <c r="S18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="n">
         <v>1</v>
@@ -8759,9 +8757,7 @@
       </c>
       <c r="R120" s="2" t="inlineStr"/>
       <c r="S120" s="2" t="inlineStr"/>
-      <c r="T120" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T120" s="2" t="inlineStr"/>
       <c r="U120" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
@@ -32282,9 +32278,7 @@
       </c>
       <c r="R463" s="2" t="inlineStr"/>
       <c r="S463" s="2" t="inlineStr"/>
-      <c r="T463" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T463" s="2" t="inlineStr"/>
       <c r="U463" s="2" t="inlineStr"/>
       <c r="V463" s="2" t="inlineStr"/>
       <c r="W463" s="2" t="inlineStr"/>
@@ -36308,7 +36302,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-06 | 525 只</t>
+          <t>截至: 2026-09-07 | 525 只</t>
         </is>
       </c>
     </row>
@@ -36432,14 +36426,14 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5%。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
+          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5% 且距250日收盘高点回落≥5%(创新高处的平台突破归新高, 不算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=1.8x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
+          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (US) 2026-09-13
</commit_message>
<xml_diff>
--- a/US_Swing_Pattern.xlsx
+++ b/US_Swing_Pattern.xlsx
@@ -6134,7 +6134,7 @@
         <v>-3.2</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>13.96</v>
+        <v>13.93</v>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
       <c r="I81" s="2" t="inlineStr"/>
@@ -10678,19 +10678,19 @@
       <c r="W147" s="2" t="inlineStr"/>
       <c r="X147" s="2" t="inlineStr"/>
       <c r="Y147" s="2" t="n">
-        <v>33.91</v>
+        <v>33.66</v>
       </c>
       <c r="Z147" s="2" t="n">
-        <v>10.45</v>
+        <v>10.46</v>
       </c>
       <c r="AA147" s="2" t="n">
-        <v>9.880000000000001</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="AB147" s="2" t="n">
         <v>2.5</v>
       </c>
       <c r="AC147" s="2" t="n">
-        <v>6.9</v>
+        <v>6.91</v>
       </c>
     </row>
     <row r="148">
@@ -13412,7 +13412,7 @@
       </c>
       <c r="X187" s="2" t="inlineStr"/>
       <c r="Y187" s="2" t="n">
-        <v>22.69</v>
+        <v>22.7</v>
       </c>
       <c r="Z187" s="2" t="n">
         <v>11.89</v>
@@ -14994,7 +14994,7 @@
         <v>54.9</v>
       </c>
       <c r="G211" s="2" t="n">
-        <v>104.67</v>
+        <v>104.64</v>
       </c>
       <c r="H211" s="2" t="inlineStr"/>
       <c r="I211" s="2" t="inlineStr"/>
@@ -17391,7 +17391,7 @@
         <v>-3.3</v>
       </c>
       <c r="G246" s="2" t="n">
-        <v>-11.85</v>
+        <v>-11.88</v>
       </c>
       <c r="H246" s="2" t="inlineStr"/>
       <c r="I246" s="2" t="inlineStr"/>
@@ -22868,7 +22868,7 @@
         <v>-4.1</v>
       </c>
       <c r="G325" s="2" t="n">
-        <v>-11.93</v>
+        <v>-11.91</v>
       </c>
       <c r="H325" s="2" t="inlineStr"/>
       <c r="I325" s="2" t="inlineStr"/>
@@ -23688,7 +23688,7 @@
         <v>-15.9</v>
       </c>
       <c r="G337" s="2" t="n">
-        <v>-0.25</v>
+        <v>-0.27</v>
       </c>
       <c r="H337" s="2" t="inlineStr"/>
       <c r="I337" s="2" t="inlineStr"/>
@@ -23873,7 +23873,7 @@
         </is>
       </c>
       <c r="C340" s="2" t="n">
-        <v>116.165</v>
+        <v>116.17</v>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
@@ -23918,16 +23918,16 @@
         <v>47.56</v>
       </c>
       <c r="Z340" s="2" t="n">
-        <v>14.29</v>
+        <v>14.3</v>
       </c>
       <c r="AA340" s="2" t="n">
         <v>14.68</v>
       </c>
       <c r="AB340" s="2" t="n">
-        <v>-1.49</v>
+        <v>-1.48</v>
       </c>
       <c r="AC340" s="2" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="341">
@@ -26026,7 +26026,7 @@
         <v>-28.1</v>
       </c>
       <c r="G371" s="2" t="n">
-        <v>1.08</v>
+        <v>1.05</v>
       </c>
       <c r="H371" s="2" t="inlineStr">
         <is>
@@ -34651,7 +34651,7 @@
         <v>-12.1</v>
       </c>
       <c r="G498" s="2" t="n">
-        <v>9.529999999999999</v>
+        <v>9.48</v>
       </c>
       <c r="H498" s="2" t="inlineStr"/>
       <c r="I498" s="2" t="inlineStr"/>
@@ -35029,7 +35029,7 @@
         <v>-10.4</v>
       </c>
       <c r="G504" s="2" t="n">
-        <v>-17.42</v>
+        <v>-17.48</v>
       </c>
       <c r="H504" s="2" t="inlineStr"/>
       <c r="I504" s="2" t="inlineStr"/>
@@ -35407,7 +35407,7 @@
         <v>-11.8</v>
       </c>
       <c r="G510" s="2" t="n">
-        <v>-4.82</v>
+        <v>-4.76</v>
       </c>
       <c r="H510" s="2" t="inlineStr"/>
       <c r="I510" s="2" t="inlineStr"/>
@@ -36100,7 +36100,7 @@
         <v>3.4</v>
       </c>
       <c r="G521" s="2" t="n">
-        <v>-14.06</v>
+        <v>-14.09</v>
       </c>
       <c r="H521" s="2" t="inlineStr"/>
       <c r="I521" s="2" t="inlineStr"/>
@@ -36543,7 +36543,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-09-12 | 526 只</t>
+          <t>截至: 2026-09-13 | 526 只</t>
         </is>
       </c>
     </row>

</xml_diff>